<commit_message>
add positional bias manually
</commit_message>
<xml_diff>
--- a/data/output/espn/merged_formatted.xlsx
+++ b/data/output/espn/merged_formatted.xlsx
@@ -117,6 +117,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -124,9 +127,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -884,7 +884,7 @@
       <c r="F12" s="3" t="n">
         <v>48</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="8" t="n">
         <v>36</v>
       </c>
       <c r="H12" s="3" t="n">
@@ -932,7 +932,7 @@
       <c r="B14" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="9" t="n">
         <v>7</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -948,7 +948,7 @@
       <c r="F14" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="9" t="n">
         <v>53</v>
       </c>
       <c r="H14" s="3" t="n">
@@ -980,7 +980,7 @@
       <c r="F15" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="9" t="n">
         <v>48</v>
       </c>
       <c r="H15" s="3" t="n">
@@ -1044,7 +1044,7 @@
       <c r="F17" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="G17" s="9" t="n">
         <v>45</v>
       </c>
       <c r="H17" s="3" t="n">
@@ -1124,7 +1124,7 @@
       <c r="B20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="7" t="n">
         <v>17</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -1156,7 +1156,7 @@
       <c r="B21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="9" t="n">
         <v>16</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -1284,7 +1284,7 @@
       <c r="B25" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="4" t="n">
         <v>18</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1300,7 +1300,7 @@
       <c r="F25" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="9" t="n">
         <v>37</v>
       </c>
       <c r="H25" s="3" t="n">
@@ -1404,7 +1404,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -1436,7 +1436,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -1444,7 +1444,7 @@
       <c r="B30" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="9" t="n">
         <v>24</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -1500,7 +1500,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -1540,7 +1540,7 @@
       <c r="B33" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C33" s="4" t="n">
         <v>44</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1604,7 +1604,7 @@
       <c r="B35" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="C35" s="6" t="n">
         <v>38</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1636,7 +1636,7 @@
       <c r="B36" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C36" s="6" t="n">
         <v>39</v>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -1668,7 +1668,7 @@
       <c r="B37" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="C37" s="8" t="n">
+      <c r="C37" s="4" t="n">
         <v>28</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1684,7 +1684,7 @@
       <c r="F37" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="9" t="n">
         <v>29</v>
       </c>
       <c r="H37" s="3" t="n">
@@ -1732,7 +1732,7 @@
       <c r="B39" s="3" t="n">
         <v>38</v>
       </c>
-      <c r="C39" s="8" t="n">
+      <c r="C39" s="7" t="n">
         <v>29</v>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -1748,7 +1748,7 @@
       <c r="F39" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="4" t="n">
         <v>28</v>
       </c>
       <c r="H39" s="3" t="n">
@@ -1756,7 +1756,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -1764,7 +1764,7 @@
       <c r="B40" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="C40" s="11" t="n">
+      <c r="C40" s="8" t="n">
         <v>57</v>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="F40" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G40" s="8" t="n">
         <v>9</v>
       </c>
       <c r="H40" s="3" t="n">
@@ -1788,7 +1788,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -1796,7 +1796,7 @@
       <c r="B41" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="C41" s="8" t="n">
+      <c r="C41" s="9" t="n">
         <v>33</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -1844,7 +1844,7 @@
       <c r="F42" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="G42" s="6" t="n">
         <v>15</v>
       </c>
       <c r="H42" s="3" t="n">
@@ -1876,7 +1876,7 @@
       <c r="F43" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="G43" s="4" t="n">
+      <c r="G43" s="6" t="n">
         <v>15</v>
       </c>
       <c r="H43" s="3" t="n">
@@ -1892,7 +1892,7 @@
       <c r="B44" s="3" t="n">
         <v>43</v>
       </c>
-      <c r="C44" s="6" t="n">
+      <c r="C44" s="4" t="n">
         <v>51</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -2020,7 +2020,7 @@
       <c r="B48" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="C48" s="4" t="n">
+      <c r="C48" s="6" t="n">
         <v>54</v>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -2116,7 +2116,7 @@
       <c r="B51" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="C51" s="11" t="n">
+      <c r="C51" s="8" t="n">
         <v>84</v>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2148,7 +2148,7 @@
       <c r="B52" s="3" t="n">
         <v>52</v>
       </c>
-      <c r="C52" s="11" t="n">
+      <c r="C52" s="4" t="n">
         <v>79</v>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2180,7 +2180,7 @@
       <c r="B53" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="C53" s="4" t="n">
+      <c r="C53" s="6" t="n">
         <v>58</v>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -2340,7 +2340,7 @@
       <c r="B58" s="3" t="n">
         <v>58</v>
       </c>
-      <c r="C58" s="11" t="n">
+      <c r="C58" s="8" t="n">
         <v>74</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -2356,7 +2356,7 @@
       <c r="F58" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="G58" s="4" t="n">
+      <c r="G58" s="6" t="n">
         <v>5</v>
       </c>
       <c r="H58" s="3" t="n">
@@ -2372,7 +2372,7 @@
       <c r="B59" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="C59" s="4" t="n">
+      <c r="C59" s="6" t="n">
         <v>63</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="9" t="inlineStr">
+      <c r="A61" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -2436,7 +2436,7 @@
       <c r="B61" s="3" t="n">
         <v>61</v>
       </c>
-      <c r="C61" s="11" t="n">
+      <c r="C61" s="4" t="n">
         <v>77</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -2452,7 +2452,7 @@
       <c r="F61" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="G61" s="4" t="n">
+      <c r="G61" s="6" t="n">
         <v>4</v>
       </c>
       <c r="H61" s="3" t="n">
@@ -2460,7 +2460,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="10" t="inlineStr">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -2492,7 +2492,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="A63" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -2500,7 +2500,7 @@
       <c r="B63" s="3" t="n">
         <v>63</v>
       </c>
-      <c r="C63" s="11" t="n">
+      <c r="C63" s="8" t="n">
         <v>106</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -2628,7 +2628,7 @@
       <c r="B67" s="3" t="n">
         <v>67</v>
       </c>
-      <c r="C67" s="4" t="n">
+      <c r="C67" s="9" t="n">
         <v>61</v>
       </c>
       <c r="D67" s="3" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="9" t="inlineStr">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -2692,7 +2692,7 @@
       <c r="B69" s="3" t="n">
         <v>69</v>
       </c>
-      <c r="C69" s="11" t="n">
+      <c r="C69" s="4" t="n">
         <v>93</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -2788,7 +2788,7 @@
       <c r="B72" s="3" t="n">
         <v>72</v>
       </c>
-      <c r="C72" s="4" t="n">
+      <c r="C72" s="9" t="n">
         <v>67</v>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -2820,7 +2820,7 @@
       <c r="B73" s="3" t="n">
         <v>73</v>
       </c>
-      <c r="C73" s="11" t="n">
+      <c r="C73" s="8" t="n">
         <v>98</v>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
       <c r="F73" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="G73" s="4" t="n">
+      <c r="G73" s="6" t="n">
         <v>2</v>
       </c>
       <c r="H73" s="3" t="n">
@@ -2852,7 +2852,7 @@
       <c r="B74" s="3" t="n">
         <v>74</v>
       </c>
-      <c r="C74" s="7" t="n">
+      <c r="C74" s="4" t="n">
         <v>59</v>
       </c>
       <c r="D74" s="3" t="inlineStr">
@@ -2916,7 +2916,7 @@
       <c r="B76" s="3" t="n">
         <v>76</v>
       </c>
-      <c r="C76" s="11" t="n">
+      <c r="C76" s="8" t="n">
         <v>105</v>
       </c>
       <c r="D76" s="3" t="inlineStr">
@@ -2948,7 +2948,7 @@
       <c r="B77" s="3" t="n">
         <v>77</v>
       </c>
-      <c r="C77" s="8" t="n">
+      <c r="C77" s="4" t="n">
         <v>64</v>
       </c>
       <c r="D77" s="3" t="inlineStr">
@@ -3076,7 +3076,7 @@
       <c r="B81" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="C81" s="4" t="n">
+      <c r="C81" s="7" t="n">
         <v>72</v>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -3108,7 +3108,7 @@
       <c r="B82" s="3" t="n">
         <v>82</v>
       </c>
-      <c r="C82" s="11" t="n">
+      <c r="C82" s="4" t="n">
         <v>109</v>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="9" t="inlineStr">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -3164,7 +3164,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="9" t="inlineStr">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -3172,7 +3172,7 @@
       <c r="B84" s="3" t="n">
         <v>84</v>
       </c>
-      <c r="C84" s="11" t="n">
+      <c r="C84" s="8" t="n">
         <v>127</v>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="9" t="inlineStr">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -3228,7 +3228,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="9" t="inlineStr">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -3236,7 +3236,7 @@
       <c r="B86" s="3" t="n">
         <v>86</v>
       </c>
-      <c r="C86" s="11" t="n">
+      <c r="C86" s="4" t="n">
         <v>119</v>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -3260,7 +3260,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="10" t="inlineStr">
+      <c r="A87" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3292,7 +3292,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="10" t="inlineStr">
+      <c r="A88" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3324,7 +3324,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="10" t="inlineStr">
+      <c r="A89" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3396,7 +3396,7 @@
       <c r="B91" s="3" t="n">
         <v>91</v>
       </c>
-      <c r="C91" s="4" t="n">
+      <c r="C91" s="9" t="n">
         <v>87</v>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -3428,7 +3428,7 @@
       <c r="B92" s="3" t="n">
         <v>92</v>
       </c>
-      <c r="C92" s="11" t="n">
+      <c r="C92" s="8" t="n">
         <v>155</v>
       </c>
       <c r="D92" s="3" t="inlineStr">
@@ -3460,7 +3460,7 @@
       <c r="B93" s="3" t="n">
         <v>93</v>
       </c>
-      <c r="C93" s="11" t="n">
+      <c r="C93" s="4" t="n">
         <v>110</v>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -3620,7 +3620,7 @@
       <c r="B98" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="C98" s="7" t="n">
+      <c r="C98" s="9" t="n">
         <v>70</v>
       </c>
       <c r="D98" s="3" t="inlineStr">
@@ -3652,7 +3652,7 @@
       <c r="B99" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="C99" s="7" t="n">
+      <c r="C99" s="4" t="n">
         <v>75</v>
       </c>
       <c r="D99" s="3" t="inlineStr">
@@ -3684,7 +3684,7 @@
       <c r="B100" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="C100" s="4" t="n">
+      <c r="C100" s="8" t="n">
         <v>113</v>
       </c>
       <c r="D100" s="3" t="inlineStr">
@@ -3716,7 +3716,7 @@
       <c r="B101" s="3" t="n">
         <v>101</v>
       </c>
-      <c r="C101" s="8" t="n">
+      <c r="C101" s="4" t="n">
         <v>82</v>
       </c>
       <c r="D101" s="3" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="10" t="inlineStr">
+      <c r="A103" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3780,7 +3780,7 @@
       <c r="B103" s="3" t="n">
         <v>103</v>
       </c>
-      <c r="C103" s="4" t="n">
+      <c r="C103" s="8" t="n">
         <v>116</v>
       </c>
       <c r="D103" s="3" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="10" t="inlineStr">
+      <c r="A104" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3836,7 +3836,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="10" t="inlineStr">
+      <c r="A105" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3868,7 +3868,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="inlineStr">
+      <c r="A106" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -3940,7 +3940,7 @@
       <c r="B108" s="3" t="n">
         <v>108</v>
       </c>
-      <c r="C108" s="7" t="n">
+      <c r="C108" s="4" t="n">
         <v>83</v>
       </c>
       <c r="D108" s="3" t="inlineStr">
@@ -3972,7 +3972,7 @@
       <c r="B109" s="3" t="n">
         <v>109</v>
       </c>
-      <c r="C109" s="7" t="n">
+      <c r="C109" s="9" t="n">
         <v>81</v>
       </c>
       <c r="D109" s="3" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="9" t="inlineStr">
+      <c r="A113" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4100,7 +4100,7 @@
       <c r="B113" s="3" t="n">
         <v>113</v>
       </c>
-      <c r="C113" s="4" t="n">
+      <c r="C113" s="7" t="n">
         <v>100</v>
       </c>
       <c r="D113" s="3" t="inlineStr">
@@ -4132,7 +4132,7 @@
       <c r="B114" s="3" t="n">
         <v>114</v>
       </c>
-      <c r="C114" s="11" t="n">
+      <c r="C114" s="4" t="n">
         <v>163</v>
       </c>
       <c r="D114" s="3" t="inlineStr">
@@ -4196,7 +4196,7 @@
       <c r="B116" s="3" t="n">
         <v>116</v>
       </c>
-      <c r="C116" s="11" t="n">
+      <c r="C116" s="4" t="n">
         <v>150</v>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -4228,7 +4228,7 @@
       <c r="B117" s="3" t="n">
         <v>117</v>
       </c>
-      <c r="C117" s="11" t="n">
+      <c r="C117" s="4" t="n">
         <v>153</v>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -4260,7 +4260,7 @@
       <c r="B118" s="3" t="n">
         <v>118</v>
       </c>
-      <c r="C118" s="11" t="n">
+      <c r="C118" s="4" t="n">
         <v>157</v>
       </c>
       <c r="D118" s="3" t="inlineStr">
@@ -4292,7 +4292,7 @@
       <c r="B119" s="3" t="n">
         <v>119</v>
       </c>
-      <c r="C119" s="11" t="n">
+      <c r="C119" s="4" t="n">
         <v>164</v>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="10" t="inlineStr">
+      <c r="A121" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -4380,7 +4380,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="10" t="inlineStr">
+      <c r="A122" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -4412,7 +4412,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="10" t="inlineStr">
+      <c r="A123" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -4444,7 +4444,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="10" t="inlineStr">
+      <c r="A124" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -4476,7 +4476,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="9" t="inlineStr">
+      <c r="A125" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4484,7 +4484,7 @@
       <c r="B125" s="3" t="n">
         <v>125</v>
       </c>
-      <c r="C125" s="8" t="n">
+      <c r="C125" s="7" t="n">
         <v>101</v>
       </c>
       <c r="D125" s="3" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="9" t="inlineStr">
+      <c r="A126" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4540,7 +4540,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="9" t="inlineStr">
+      <c r="A127" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4572,7 +4572,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="9" t="inlineStr">
+      <c r="A128" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4580,7 +4580,7 @@
       <c r="B128" s="3" t="n">
         <v>128</v>
       </c>
-      <c r="C128" s="4" t="n">
+      <c r="C128" s="9" t="n">
         <v>120</v>
       </c>
       <c r="D128" s="3" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="9" t="inlineStr">
+      <c r="A129" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4644,7 +4644,7 @@
       <c r="B130" s="3" t="n">
         <v>130</v>
       </c>
-      <c r="C130" s="11" t="n">
+      <c r="C130" s="4" t="n">
         <v>151</v>
       </c>
       <c r="D130" s="3" t="inlineStr">
@@ -4676,7 +4676,7 @@
       <c r="B131" s="3" t="n">
         <v>131</v>
       </c>
-      <c r="C131" s="11" t="n">
+      <c r="C131" s="4" t="n">
         <v>162</v>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -4740,7 +4740,7 @@
       <c r="B133" s="3" t="n">
         <v>133</v>
       </c>
-      <c r="C133" s="4" t="n">
+      <c r="C133" s="7" t="n">
         <v>117</v>
       </c>
       <c r="D133" s="3" t="inlineStr">
@@ -4804,7 +4804,7 @@
       <c r="B135" s="3" t="n">
         <v>135</v>
       </c>
-      <c r="C135" s="11" t="n">
+      <c r="C135" s="4" t="n">
         <v>188</v>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -4836,7 +4836,7 @@
       <c r="B136" s="3" t="n">
         <v>136</v>
       </c>
-      <c r="C136" s="11" t="n">
+      <c r="C136" s="8" t="n">
         <v>221</v>
       </c>
       <c r="D136" s="3" t="inlineStr">
@@ -4868,7 +4868,7 @@
       <c r="B137" s="3" t="n">
         <v>137</v>
       </c>
-      <c r="C137" s="11" t="n">
+      <c r="C137" s="8" t="n">
         <v>173</v>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -4964,7 +4964,7 @@
       <c r="B140" s="3" t="n">
         <v>140</v>
       </c>
-      <c r="C140" s="7" t="n">
+      <c r="C140" s="4" t="n">
         <v>111</v>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="9" t="inlineStr">
+      <c r="A141" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -4996,7 +4996,7 @@
       <c r="B141" s="3" t="n">
         <v>141</v>
       </c>
-      <c r="C141" s="11" t="n">
+      <c r="C141" s="4" t="n">
         <v>169</v>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="9" t="inlineStr">
+      <c r="A142" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -5028,7 +5028,7 @@
       <c r="B142" s="3" t="n">
         <v>142</v>
       </c>
-      <c r="C142" s="4" t="n">
+      <c r="C142" s="9" t="n">
         <v>134</v>
       </c>
       <c r="D142" s="3" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="10" t="inlineStr">
+      <c r="A143" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -5084,7 +5084,7 @@
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="10" t="inlineStr">
+      <c r="A144" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -5092,7 +5092,7 @@
       <c r="B144" s="3" t="n">
         <v>144</v>
       </c>
-      <c r="C144" s="11" t="n">
+      <c r="C144" s="8" t="n">
         <v>176</v>
       </c>
       <c r="D144" s="3" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="A145" s="10" t="inlineStr">
+      <c r="A145" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -5156,7 +5156,7 @@
       <c r="B146" s="3" t="n">
         <v>146</v>
       </c>
-      <c r="C146" s="11" t="n">
+      <c r="C146" s="4" t="n">
         <v>165</v>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -5220,7 +5220,7 @@
       <c r="B148" s="3" t="n">
         <v>148</v>
       </c>
-      <c r="C148" s="4" t="n">
+      <c r="C148" s="9" t="n">
         <v>142</v>
       </c>
       <c r="D148" s="3" t="inlineStr">
@@ -5252,7 +5252,7 @@
       <c r="B149" s="3" t="n">
         <v>149</v>
       </c>
-      <c r="C149" s="4" t="n">
+      <c r="C149" s="7" t="n">
         <v>135</v>
       </c>
       <c r="D149" s="3" t="inlineStr">
@@ -5284,7 +5284,7 @@
       <c r="B150" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="C150" s="4" t="n">
+      <c r="C150" s="7" t="n">
         <v>137</v>
       </c>
       <c r="D150" s="3" t="inlineStr">
@@ -5316,7 +5316,7 @@
       <c r="B151" s="3" t="n">
         <v>151</v>
       </c>
-      <c r="C151" s="11" t="n">
+      <c r="C151" s="4" t="n">
         <v>195</v>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -5348,7 +5348,7 @@
       <c r="B152" s="3" t="n">
         <v>152</v>
       </c>
-      <c r="C152" s="11" t="n">
+      <c r="C152" s="6" t="n">
         <v>218</v>
       </c>
       <c r="D152" s="3" t="inlineStr">
@@ -5380,7 +5380,7 @@
       <c r="B153" s="3" t="n">
         <v>153</v>
       </c>
-      <c r="C153" s="11" t="n">
+      <c r="C153" s="6" t="n">
         <v>184</v>
       </c>
       <c r="D153" s="3" t="inlineStr">
@@ -5412,7 +5412,7 @@
       <c r="B154" s="3" t="n">
         <v>154</v>
       </c>
-      <c r="C154" s="8" t="n">
+      <c r="C154" s="4" t="n">
         <v>124</v>
       </c>
       <c r="D154" s="3" t="inlineStr">
@@ -5476,7 +5476,7 @@
       <c r="B156" s="3" t="n">
         <v>156</v>
       </c>
-      <c r="C156" s="7" t="n">
+      <c r="C156" s="9" t="n">
         <v>112</v>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -5508,7 +5508,7 @@
       <c r="B157" s="3" t="n">
         <v>158</v>
       </c>
-      <c r="C157" s="11" t="n">
+      <c r="C157" s="6" t="n">
         <v>192</v>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -5540,7 +5540,7 @@
       <c r="B158" s="3" t="n">
         <v>159</v>
       </c>
-      <c r="C158" s="11" t="n">
+      <c r="C158" s="6" t="n">
         <v>180</v>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -5700,7 +5700,7 @@
       <c r="B163" s="3" t="n">
         <v>164</v>
       </c>
-      <c r="C163" s="11" t="n">
+      <c r="C163" s="6" t="n">
         <v>219</v>
       </c>
       <c r="D163" s="3" t="inlineStr">
@@ -5724,7 +5724,7 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="9" t="inlineStr">
+      <c r="A164" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -5756,7 +5756,7 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="9" t="inlineStr">
+      <c r="A165" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -5764,7 +5764,7 @@
       <c r="B165" s="3" t="n">
         <v>166</v>
       </c>
-      <c r="C165" s="11" t="n">
+      <c r="C165" s="6" t="n">
         <v>207</v>
       </c>
       <c r="D165" s="3" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="9" t="inlineStr">
+      <c r="A166" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -5820,7 +5820,7 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="9" t="inlineStr">
+      <c r="A167" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -5988,7 +5988,7 @@
       <c r="B172" s="3" t="n">
         <v>197</v>
       </c>
-      <c r="C172" s="11" t="n">
+      <c r="C172" s="4" t="n">
         <v>223</v>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="10" t="inlineStr">
+      <c r="A173" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6044,7 +6044,7 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="10" t="inlineStr">
+      <c r="A174" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6052,7 +6052,7 @@
       <c r="B174" s="3" t="n">
         <v>199</v>
       </c>
-      <c r="C174" s="8" t="n">
+      <c r="C174" s="9" t="n">
         <v>161</v>
       </c>
       <c r="D174" s="3" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="10" t="inlineStr">
+      <c r="A175" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6084,7 +6084,7 @@
       <c r="B175" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="C175" s="8" t="n">
+      <c r="C175" s="9" t="n">
         <v>147</v>
       </c>
       <c r="D175" s="3" t="inlineStr">
@@ -6116,7 +6116,7 @@
       <c r="B176" s="3" t="n">
         <v>201</v>
       </c>
-      <c r="C176" s="8" t="n">
+      <c r="C176" s="9" t="n">
         <v>149</v>
       </c>
       <c r="D176" s="3" t="inlineStr">
@@ -6180,7 +6180,7 @@
       <c r="B178" s="3" t="n">
         <v>203</v>
       </c>
-      <c r="C178" s="8" t="n">
+      <c r="C178" s="9" t="n">
         <v>144</v>
       </c>
       <c r="D178" s="3" t="inlineStr">
@@ -6268,7 +6268,7 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="9" t="inlineStr">
+      <c r="A181" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -6276,7 +6276,7 @@
       <c r="B181" s="3" t="n">
         <v>206</v>
       </c>
-      <c r="C181" s="8" t="n">
+      <c r="C181" s="9" t="n">
         <v>170</v>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -6300,7 +6300,7 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="9" t="inlineStr">
+      <c r="A182" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -6340,7 +6340,7 @@
       <c r="B183" s="3" t="n">
         <v>208</v>
       </c>
-      <c r="C183" s="8" t="n">
+      <c r="C183" s="9" t="n">
         <v>140</v>
       </c>
       <c r="D183" s="3" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="9" t="inlineStr">
+      <c r="A190" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -6588,7 +6588,7 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="9" t="inlineStr">
+      <c r="A191" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -6620,7 +6620,7 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="9" t="inlineStr">
+      <c r="A192" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -6652,7 +6652,7 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="10" t="inlineStr">
+      <c r="A193" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6660,7 +6660,7 @@
       <c r="B193" s="3" t="n">
         <v>218</v>
       </c>
-      <c r="C193" s="8" t="n">
+      <c r="C193" s="9" t="n">
         <v>133</v>
       </c>
       <c r="D193" s="3" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="10" t="inlineStr">
+      <c r="A194" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6692,7 +6692,7 @@
       <c r="B194" s="3" t="n">
         <v>219</v>
       </c>
-      <c r="C194" s="8" t="n">
+      <c r="C194" s="9" t="n">
         <v>154</v>
       </c>
       <c r="D194" s="3" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="10" t="inlineStr">
+      <c r="A195" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -6724,7 +6724,7 @@
       <c r="B195" s="3" t="n">
         <v>220</v>
       </c>
-      <c r="C195" s="8" t="n">
+      <c r="C195" s="9" t="n">
         <v>175</v>
       </c>
       <c r="D195" s="3" t="inlineStr">
@@ -6788,7 +6788,7 @@
       <c r="B197" s="3" t="n">
         <v>222</v>
       </c>
-      <c r="C197" s="8" t="n">
+      <c r="C197" s="9" t="n">
         <v>152</v>
       </c>
       <c r="D197" s="3" t="inlineStr">
@@ -6884,7 +6884,7 @@
       <c r="B200" s="3" t="n">
         <v>225</v>
       </c>
-      <c r="C200" s="8" t="n">
+      <c r="C200" s="9" t="n">
         <v>156</v>
       </c>
       <c r="D200" s="3" t="inlineStr">
@@ -6916,7 +6916,7 @@
       <c r="B201" s="3" t="n">
         <v>226</v>
       </c>
-      <c r="C201" s="8" t="n">
+      <c r="C201" s="9" t="n">
         <v>189</v>
       </c>
       <c r="D201" s="3" t="inlineStr">
@@ -6976,7 +6976,7 @@
       <c r="B203" s="3" t="n">
         <v>229</v>
       </c>
-      <c r="C203" s="8" t="n">
+      <c r="C203" s="9" t="n">
         <v>183</v>
       </c>
       <c r="D203" s="3" t="inlineStr">
@@ -7136,7 +7136,7 @@
       <c r="B208" s="3" t="n">
         <v>239</v>
       </c>
-      <c r="C208" s="8" t="n">
+      <c r="C208" s="9" t="n">
         <v>187</v>
       </c>
       <c r="D208" s="3" t="inlineStr">
@@ -7384,7 +7384,7 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="9" t="inlineStr">
+      <c r="A216" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -7416,7 +7416,7 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="9" t="inlineStr">
+      <c r="A217" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -7448,7 +7448,7 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="9" t="inlineStr">
+      <c r="A218" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -7488,7 +7488,7 @@
       <c r="B219" s="3" t="n">
         <v>261</v>
       </c>
-      <c r="C219" s="8" t="n">
+      <c r="C219" s="9" t="n">
         <v>191</v>
       </c>
       <c r="D219" s="3" t="inlineStr">
@@ -7648,7 +7648,7 @@
       <c r="B224" s="3" t="n">
         <v>266</v>
       </c>
-      <c r="C224" s="8" t="n">
+      <c r="C224" s="9" t="n">
         <v>177</v>
       </c>
       <c r="D224" s="3" t="inlineStr">
@@ -7672,7 +7672,7 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="10" t="inlineStr">
+      <c r="A225" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -7680,7 +7680,7 @@
       <c r="B225" s="3" t="n">
         <v>267</v>
       </c>
-      <c r="C225" s="8" t="n">
+      <c r="C225" s="9" t="n">
         <v>160</v>
       </c>
       <c r="D225" s="3" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="10" t="inlineStr">
+      <c r="A226" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -7712,7 +7712,7 @@
       <c r="B226" s="3" t="n">
         <v>268</v>
       </c>
-      <c r="C226" s="8" t="n">
+      <c r="C226" s="9" t="n">
         <v>194</v>
       </c>
       <c r="D226" s="3" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="10" t="inlineStr">
+      <c r="A227" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -7744,7 +7744,7 @@
       <c r="B227" s="3" t="n">
         <v>269</v>
       </c>
-      <c r="C227" s="8" t="n">
+      <c r="C227" s="9" t="n">
         <v>186</v>
       </c>
       <c r="D227" s="3" t="inlineStr">
@@ -7768,7 +7768,7 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="10" t="inlineStr">
+      <c r="A228" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -7808,7 +7808,7 @@
       <c r="B229" s="3" t="n">
         <v>271</v>
       </c>
-      <c r="C229" s="8" t="n">
+      <c r="C229" s="9" t="n">
         <v>193</v>
       </c>
       <c r="D229" s="3" t="inlineStr">
@@ -7840,7 +7840,7 @@
       <c r="B230" s="3" t="n">
         <v>272</v>
       </c>
-      <c r="C230" s="8" t="n">
+      <c r="C230" s="9" t="n">
         <v>179</v>
       </c>
       <c r="D230" s="3" t="inlineStr">
@@ -7968,7 +7968,7 @@
       <c r="B234" s="3" t="n">
         <v>283</v>
       </c>
-      <c r="C234" s="8" t="n">
+      <c r="C234" s="9" t="n">
         <v>197</v>
       </c>
       <c r="D234" s="3" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="9" t="inlineStr">
+      <c r="A235" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8000,7 +8000,7 @@
       <c r="B235" s="3" t="n">
         <v>289</v>
       </c>
-      <c r="C235" s="8" t="n">
+      <c r="C235" s="9" t="n">
         <v>172</v>
       </c>
       <c r="D235" s="3" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="9" t="inlineStr">
+      <c r="A236" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8032,7 +8032,7 @@
       <c r="B236" s="3" t="n">
         <v>290</v>
       </c>
-      <c r="C236" s="8" t="n">
+      <c r="C236" s="9" t="n">
         <v>167</v>
       </c>
       <c r="D236" s="3" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="9" t="inlineStr">
+      <c r="A237" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8064,7 +8064,7 @@
       <c r="B237" s="3" t="n">
         <v>291</v>
       </c>
-      <c r="C237" s="8" t="n">
+      <c r="C237" s="9" t="n">
         <v>199</v>
       </c>
       <c r="D237" s="3" t="inlineStr">
@@ -8088,7 +8088,7 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="9" t="inlineStr">
+      <c r="A238" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8120,7 +8120,7 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="10" t="inlineStr">
+      <c r="A239" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8128,7 +8128,7 @@
       <c r="B239" s="3" t="n">
         <v>296</v>
       </c>
-      <c r="C239" s="8" t="n">
+      <c r="C239" s="9" t="n">
         <v>185</v>
       </c>
       <c r="D239" s="3" t="inlineStr">
@@ -8152,7 +8152,7 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="10" t="inlineStr">
+      <c r="A240" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8160,7 +8160,7 @@
       <c r="B240" s="3" t="n">
         <v>301</v>
       </c>
-      <c r="C240" s="8" t="n">
+      <c r="C240" s="9" t="n">
         <v>178</v>
       </c>
       <c r="D240" s="3" t="inlineStr">
@@ -8184,7 +8184,7 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="10" t="inlineStr">
+      <c r="A241" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8280,7 +8280,7 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="9" t="inlineStr">
+      <c r="A244" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8312,7 +8312,7 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="9" t="inlineStr">
+      <c r="A245" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8344,7 +8344,7 @@
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="9" t="inlineStr">
+      <c r="A246" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8376,7 +8376,7 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="10" t="inlineStr">
+      <c r="A247" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8408,7 +8408,7 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="10" t="inlineStr">
+      <c r="A248" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8440,7 +8440,7 @@
       </c>
     </row>
     <row r="249">
-      <c r="A249" s="10" t="inlineStr">
+      <c r="A249" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8472,7 +8472,7 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="10" t="inlineStr">
+      <c r="A250" s="11" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
@@ -8504,7 +8504,7 @@
       </c>
     </row>
     <row r="251">
-      <c r="A251" s="9" t="inlineStr">
+      <c r="A251" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8536,7 +8536,7 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="9" t="inlineStr">
+      <c r="A252" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8568,7 +8568,7 @@
       </c>
     </row>
     <row r="253">
-      <c r="A253" s="9" t="inlineStr">
+      <c r="A253" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8600,7 +8600,7 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="9" t="inlineStr">
+      <c r="A254" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>
@@ -8632,7 +8632,7 @@
       </c>
     </row>
     <row r="255">
-      <c r="A255" s="9" t="inlineStr">
+      <c r="A255" s="10" t="inlineStr">
         <is>
           <t>TE</t>
         </is>

</xml_diff>